<commit_message>
Atualiza base SQDCP FMDS
</commit_message>
<xml_diff>
--- a/data/sqdcp_base.xlsx
+++ b/data/sqdcp_base.xlsx
@@ -629,7 +629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -656,6 +656,31 @@
       <c r="E1" t="inlineStr">
         <is>
           <t>status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Acidentes</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>treinametno mensal relacionado a acidentes</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Luis Fernando</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>46203</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Aberta</t>
         </is>
       </c>
     </row>

</xml_diff>